<commit_message>
quede en ficha nueva para la vista table
</commit_message>
<xml_diff>
--- a/juicios_pendientes.xlsx
+++ b/juicios_pendientes.xlsx
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45390</v>
+        <v>45391</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2041211</t>
+          <t>5050505</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se soluciono error al consultar fichas por primera vez
</commit_message>
<xml_diff>
--- a/juicios_pendientes.xlsx
+++ b/juicios_pendientes.xlsx
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45391</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5050505</t>
+          <t>2041211</t>
         </is>
       </c>
     </row>

</xml_diff>